<commit_message>
Turned book object into data class, and added pagentation via next button.
</commit_message>
<xml_diff>
--- a/TrialRun.xlsx
+++ b/TrialRun.xlsx
@@ -12,11 +12,6 @@
     <sheet name="Books, page 3" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Books, page 4" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Books, page 5" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Books, page 6" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Books, page 7" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Books, page 8" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Books, page 9" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Books, page 10" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -682,272 +677,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Modern Romance</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£28.26</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Miss Peregrine’s Home for Peculiar Children (Miss Peregrine’s Peculiar Children #1)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£10.76</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Louisa: The Extraordinary Life of Mrs. Adams</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£16.85</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Little Red</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£13.47</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Library of Souls (Miss Peregrine’s Peculiar Children #3)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£48.56</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Large Print Heart of the Pride</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£19.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>I Had a Nice Time And Other Lies...: How to find love &amp; sh*t like that</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£57.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Hollow City (Miss Peregrine’s Peculiar Children #2)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£42.98</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Grumbles</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£22.16</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Full Moon over Noah’s Ark: An Odyssey to Mount Ararat and Beyond</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£49.43</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Frostbite (Vampire Academy #2)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£29.99</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Follow You Home</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>£21.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>First Steps for New Christians (Print Edition)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>£29.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Finders Keepers (Bill Hodges Trilogy #2)</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>£53.53</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Fables, Vol. 1: Legends in Exile (Fables #1)</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>£41.62</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Eureka Trivia 6.0</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>£54.59</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Drive: The Surprising Truth About What Motivates Us</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>£34.95</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Done Rubbed Out (Reightman &amp; Bailey #1)</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>£37.72</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Doing It Over (Most Likely To #1)</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>£35.61</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Deliciously Ella Every Day: Quick and Easy Recipes for Gluten-Free Snacks, Packed Lunches, and Simple Meals</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>£42.16</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2010,1068 +1739,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Immunity: How Elie Metchnikoff Changed the Course of Modern Medicine</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£57.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>I Hate Fairyland, Vol. 1: Madly Ever After (I Hate Fairyland (Compilations) #1-5)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£29.17</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>I am a Hero Omnibus Volume 1</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£54.63</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>How to Be Miserable: 40 Strategies You Already Use</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£46.03</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Her Backup Boyfriend (The Sorensen Family #1)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£33.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Giant Days, Vol. 2 (Giant Days #5-8)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£22.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Forever and Forever: The Courtship of Henry Longfellow and Fanny Appleton</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£29.69</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>First and First (Five Boroughs #3)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£15.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Fifty Shades Darker (Fifty Shades #2)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£21.96</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Everydata: The Misinformation Hidden in the Little Data You Consume Every Day</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£54.35</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Don't Be a Jerk: And Other Practical Advice from Dogen, Japan's Greatest Zen Master</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£37.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Danganronpa Volume 1</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>£51.99</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Crown of Midnight (Throne of Glass #2)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>£43.29</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Codename Baboushka, Volume 1: The Conclave of Death</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>£36.72</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Camp Midnight</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>£17.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Call the Nurse: True Stories of a Country Nurse on a Scottish Isle</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>£29.14</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Burning</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>£28.81</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Bossypants</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>£49.46</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Bitch Planet, Vol. 1: Extraordinary Machine (Bitch Planet (Collected Editions))</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>£37.92</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Avatar: The Last Airbender: Smoke and Shadow, Part 3 (Smoke and Shadow #3)</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>£28.09</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Algorithms to Live By: The Computer Science of Human Decisions</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£30.81</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>A World of Flavor: Your Gluten Free Passport</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£42.95</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>A Piece of Sky, a Grain of Rice: A Memoir in Four Meditations</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£56.76</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>A Murder in Time</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£16.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>A Flight of Arrows (The Pathfinders #2)</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£55.53</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>A Fierce and Subtle Poison</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£28.13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>A Court of Thorns and Roses (A Court of Thorns and Roses #1)</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£52.37</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>(Un)Qualified: How God Uses Broken People to Do Big Things</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£54.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>You Are What You Love: The Spiritual Power of Habit</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£21.87</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>William Shakespeare's Star Wars: Verily, A New Hope (William Shakespeare's Star Wars #4)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£43.30</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tuesday Nights in 1980</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£21.04</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Tracing Numbers on a Train</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>£41.60</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Throne of Glass (Throne of Glass #1)</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>£35.07</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Thomas Jefferson and the Tripoli Pirates: The Forgotten War That Changed American History</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>£59.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Thirteen Reasons Why</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>£52.72</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>The White Cat and the Monk: A Retelling of the Poem “Pangur Bán”</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>£58.08</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>The Wedding Dress</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>£24.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>The Vacationers</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>£42.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>The Third Wave: An Entrepreneur’s Vision of the Future</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>£12.61</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>The Stranger</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>£17.44</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>The Shadow Hero (The Shadow Hero)</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£33.14</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>The Secret (The Secret #1)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£27.37</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>The Regional Office Is Under Attack!</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£51.36</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>The Psychopath Test: A Journey Through the Madness Industry</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£36.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>The Project</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£10.65</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>The Power of Now: A Guide to Spiritual Enlightenment</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£43.54</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>The Omnivore's Dilemma: A Natural History of Four Meals</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£38.21</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>The Nerdy Nummies Cookbook: Sweet Treats for the Geek in All of Us</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£37.34</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>The Murder of Roger Ackroyd (Hercule Poirot #4)</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£44.10</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>The Mistake (Off-Campus #2)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£43.29</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>The Matchmaker's Playbook (Wingmen Inc. #1)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£55.85</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>The Love and Lemons Cookbook: An Apple-to-Zucchini Celebration of Impromptu Cooking</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>£37.60</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>The Long Shadow of Small Ghosts: Murder and Memory in an American City</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>£10.97</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>The Kite Runner</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>£41.82</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>The House by the Lake</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>£36.95</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>The Glittering Court (The Glittering Court #1)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>£44.28</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>The Girl on the Train</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>£55.02</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>The Genius of Birds</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>£17.24</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>The Emerald Mystery</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>£23.15</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>The Cookies &amp; Cups Cookbook: 125+ sweet &amp; savory recipes reminding you to Always Eat Dessert First</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>£41.25</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>The Bridge to Consciousness: I'm Writing the Bridge Between Science and Our Old and New Beliefs.</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>£32.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>The Artist's Way: A Spiritual Path to Higher Creativity</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>£38.49</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>The Art of War</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>£33.34</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>The Argonauts</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>£10.93</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>The 10% Entrepreneur: Live Your Startup Dream Without Quitting Your Day Job</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>£27.55</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Suddenly in Love (Lake Haven #1)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>£55.99</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Something More Than This</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>£16.24</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Soft Apocalypse</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>£26.12</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>So You've Been Publicly Shamed</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>£12.23</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Shoe Dog: A Memoir by the Creator of NIKE</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>£23.99</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Shobu Samurai, Project Aryoku (#3)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>£29.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Secrets and Lace (Fatal Hearts #1)</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>£20.27</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Scarlett Epstein Hates It Here</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>£43.55</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Romero and Juliet: A Tragic Tale of Love and Zombies</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>£36.94</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Redeeming Love</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>£20.47</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Poses for Artists Volume 1 - Dynamic and Sitting Poses: An Essential Reference for Figure Drawing and the Human Form</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>£41.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Poems That Make Grown Women Cry</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>£14.19</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Nightingale, Sing</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>£38.28</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Night Sky with Exit Wounds</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>£41.05</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Mrs. Houdini</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>£30.25</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>